<commit_message>
ml: update fsch forms
</commit_message>
<xml_diff>
--- a/SCH-STH/Impact assessments/Mali/2025/ml_sch_sth_impact_2501_2_child.xlsx
+++ b/SCH-STH/Impact assessments/Mali/2025/ml_sch_sth_impact_2501_2_child.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\SCH-STH\Impact assessments\Mali\2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3710B4C-E8C7-4682-B5C2-4990079139DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FC967F6-D688-4691-8CE0-423B048FE1B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -563,12 +563,6 @@
     <t>Veuillez enregistrer le code unique de l’enfant et des échantillons de labo </t>
   </si>
   <si>
-    <t>ml_sch_sth_impact_2501_2_child_v2_1</t>
-  </si>
-  <si>
-    <t>(2025 Jan) - 2. SCH/STH – Enrôlement V2.1</t>
-  </si>
-  <si>
     <t>ml_ia_e_250121</t>
   </si>
   <si>
@@ -584,9 +578,6 @@
     <t>not(selected(${C3}, ${p_code_id}))</t>
   </si>
   <si>
-    <t>concat(${p_recorder} , '_',  ${p_site_id} , '_',  ${p_sequential_code})</t>
-  </si>
-  <si>
     <t>p_sequential_code</t>
   </si>
   <si>
@@ -597,6 +588,15 @@
   </si>
   <si>
     <t>Cet identifiant a déjà été utilisé dans ce village.</t>
+  </si>
+  <si>
+    <t>ml_sch_sth_impact_2501_2_child_v3</t>
+  </si>
+  <si>
+    <t>(2025 Jan) - 2. SCH/STH – Enrôlement V3</t>
+  </si>
+  <si>
+    <t>concat(${p_site_id} , '_',  ${p_sequential_code})</t>
   </si>
 </sst>
 </file>
@@ -1445,7 +1445,7 @@
         <v>163</v>
       </c>
       <c r="B8" s="36" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C8" s="37" t="s">
         <v>164</v>
@@ -1504,7 +1504,7 @@
       <c r="L10" s="33"/>
       <c r="M10" s="33"/>
     </row>
-    <row r="11" spans="1:19" s="17" customFormat="1" ht="169.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" s="17" customFormat="1" ht="188.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>19</v>
       </c>
@@ -1560,15 +1560,15 @@
       <c r="R12" s="30"/>
       <c r="S12" s="31"/>
     </row>
-    <row r="13" spans="1:19" s="17" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" s="17" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>29</v>
       </c>
       <c r="B13" s="25" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D13" s="10"/>
       <c r="E13" s="9"/>
@@ -1596,18 +1596,18 @@
         <v>29</v>
       </c>
       <c r="B14" s="25" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="D14" s="10"/>
       <c r="E14" s="9"/>
       <c r="F14" s="42" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="H14" s="9" t="s">
         <v>26</v>
@@ -1626,7 +1626,7 @@
       <c r="R14" s="32"/>
       <c r="S14" s="32"/>
     </row>
-    <row r="15" spans="1:19" s="17" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" s="17" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>28</v>
       </c>
@@ -1639,16 +1639,16 @@
       <c r="D15" s="10"/>
       <c r="E15" s="9"/>
       <c r="F15" s="42" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G15" s="43" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="H15" s="9" t="s">
         <v>26</v>
       </c>
       <c r="I15" s="25" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="J15" s="9" t="s">
         <v>13</v>
@@ -2683,7 +2683,7 @@
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="44.125" customWidth="1"/>
-    <col min="2" max="2" width="32.125" customWidth="1"/>
+    <col min="2" max="2" width="35.125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -2697,12 +2697,12 @@
         <v>142</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="C2" t="s">
         <v>143</v>

</xml_diff>